<commit_message>
multiple cmoiits reg parallel testing
</commit_message>
<xml_diff>
--- a/src/test/resources/TestData/testdatssheet.xlsx
+++ b/src/test/resources/TestData/testdatssheet.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dell\eclipse-workspace_TestNG_automation\TestNG_auto_framework\src\test\resources\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA686286-39A4-478B-B336-09853869C8AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75E96348-6D50-45B7-BFEC-967EDC203AED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="12240" xr2:uid="{333944E2-6ADB-4FAD-B3E5-5B3E0DB9BBEE}"/>
   </bookViews>
   <sheets>
-    <sheet name="Login" sheetId="1" r:id="rId1"/>
+    <sheet name="excelsheet" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -33,10 +33,10 @@
     <t>Password</t>
   </si>
   <si>
-    <t>ranipatange4@gmail.com</t>
+    <t>shwetasutar041@gmail.com</t>
   </si>
   <si>
-    <t>patange12@223</t>
+    <t>Ranipatange@223</t>
   </si>
 </sst>
 </file>
@@ -119,7 +119,7 @@
         <a:srgbClr val="E7E6E6"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="5B9BD5"/>
+        <a:srgbClr val="4472C4"/>
       </a:accent1>
       <a:accent2>
         <a:srgbClr val="ED7D31"/>
@@ -131,7 +131,7 @@
         <a:srgbClr val="FFC000"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4472C4"/>
+        <a:srgbClr val="5B9BD5"/>
       </a:accent5>
       <a:accent6>
         <a:srgbClr val="70AD47"/>
@@ -178,6 +178,23 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri" panose="020F0502020204030204"/>
@@ -213,6 +230,23 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -364,12 +398,12 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{321F00A1-4BCF-4F7F-AE15-354ABDD61B3D}">
   <dimension ref="A1:B2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="31.21875" customWidth="1"/>
-    <col min="2" max="2" width="24.21875" customWidth="1"/>
+    <col min="1" max="1" width="25.109375" customWidth="1"/>
+    <col min="2" max="2" width="27.77734375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
@@ -390,8 +424,8 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1" xr:uid="{62811A5B-E1B7-41C4-8ECE-A9FD60A942DF}"/>
-    <hyperlink ref="B2" r:id="rId2" xr:uid="{EA1F8931-FA7E-480D-83DE-E6B28F29D42C}"/>
+    <hyperlink ref="A2" r:id="rId1" xr:uid="{F6A36629-F422-48D2-92BE-A4D25D75E96C}"/>
+    <hyperlink ref="B2" r:id="rId2" xr:uid="{BF8449A0-9FFB-4D8E-9FA1-3C4DA05F0981}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>